<commit_message>
fix download excel logic
</commit_message>
<xml_diff>
--- a/e2e/expectedData/sub_Daftar_Transfer_Potongan.xlsx
+++ b/e2e/expectedData/sub_Daftar_Transfer_Potongan.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="28">
   <si>
     <t>DAFTAR TRANSFER POTONGAN</t>
   </si>
@@ -47,10 +47,40 @@
     <t>JUMLAH TRANSFER</t>
   </si>
   <si>
-    <t>No Data Available</t>
-  </si>
-  <si>
-    <t>DILI, 10 September 2026</t>
+    <t>TWP Deduction</t>
+  </si>
+  <si>
+    <t>$23.05</t>
+  </si>
+  <si>
+    <t>PT AZKO</t>
+  </si>
+  <si>
+    <t>Mandiri</t>
+  </si>
+  <si>
+    <t>IDP Deduction</t>
+  </si>
+  <si>
+    <t>$16.25</t>
+  </si>
+  <si>
+    <t>Heri Mulyadi</t>
+  </si>
+  <si>
+    <t>BCA</t>
+  </si>
+  <si>
+    <t>SUB TOTAL DI BANK INDONESIA</t>
+  </si>
+  <si>
+    <t>$39.30</t>
+  </si>
+  <si>
+    <t>TOTAL SETORAN POTONGAN</t>
+  </si>
+  <si>
+    <t>DILI, 11 September 2026</t>
   </si>
   <si>
     <t>Human Resource</t>
@@ -137,7 +167,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -149,7 +179,21 @@
     <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
@@ -171,7 +215,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>12</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="571500" cy="333375"/>
@@ -490,7 +534,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="true" style="0"/>
@@ -544,72 +588,133 @@
       </c>
     </row>
     <row r="6" spans="1:7">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="5">
+        <v>1</v>
+      </c>
+      <c r="B6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
+      <c r="C6" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="6">
+        <v>928379837</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="7" spans="1:7">
-      <c r="A7"/>
+      <c r="A7" s="5">
+        <v>2</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" s="6">
+        <v>233643546</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="8" spans="1:7">
-      <c r="A8" s="6" t="s">
-        <v>11</v>
+      <c r="A8" s="8" t="s">
+        <v>18</v>
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="6"/>
       <c r="D8" s="6"/>
       <c r="E8" s="6"/>
       <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
+      <c r="G8" s="9" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="9" spans="1:7">
-      <c r="A9" s="6" t="s">
-        <v>12</v>
+      <c r="A9" s="8" t="s">
+        <v>20</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
-      <c r="D9" s="6" t="s">
-        <v>13</v>
-      </c>
+      <c r="D9" s="6"/>
       <c r="E9" s="6"/>
       <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
-    </row>
-    <row r="10" spans="1:7" customHeight="1" ht="37.5">
+      <c r="G9" s="9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
       <c r="A10"/>
-      <c r="D10"/>
     </row>
     <row r="11" spans="1:7">
-      <c r="A11" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
+      <c r="A11" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" s="10"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10"/>
     </row>
     <row r="12" spans="1:7">
-      <c r="A12" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
+      <c r="A12" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="E12" s="10"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
+    </row>
+    <row r="13" spans="1:7" customHeight="1" ht="37.5">
+      <c r="A13"/>
+      <c r="D13"/>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="E14" s="10"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10"/>
     </row>
   </sheetData>
   <mergeCells>
@@ -617,18 +722,19 @@
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A3:G3"/>
     <mergeCell ref="A4:G4"/>
-    <mergeCell ref="A6:G6"/>
-    <mergeCell ref="A7:G7"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="D8:G8"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="D9:G9"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="D10:G10"/>
+    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="A10:G10"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="D11:G11"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="D12:G12"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="D13:G13"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="D14:G14"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="D15:G15"/>
   </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>